<commit_message>
NICA: cierres de la semana 12-18 oct ajustados al brief aprobado (semana foco Querida Ansiedad)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qf6tRYSFcLAZC7iH3hkQz4
</commit_message>
<xml_diff>
--- a/nica-apify/calendario/calendario-semana-2026-10-12.xlsx
+++ b/nica-apify/calendario/calendario-semana-2026-10-12.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cómo leer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Calendario" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Guion por partes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mi semana" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Podcast y YouTube" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Querido Ex" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Competencia" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Patrones de viralidad" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo leer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guion por partes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mi semana" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podcast y YouTube" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Querido Ex" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competencia" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patrones de viralidad" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Calendario'!$A$1:$AD$22</definedName>
@@ -1317,8 +1317,7 @@
 [1:20–1:40] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: una meta que se te dio cuando empezaste a actuar como si ya la tuvieras]"
 [1:40–2:21] HACKEO (hazlo conmigo) ✂️: "Hoy escribe tu propio cheque: tu nombre, una cifra realista para los próximos 12 meses y una fecha. Detrás escribe: ¿qué haría hoy la mujer que ya cobra esto? Y haz una de esas cosas hoy mismo. Repite conmigo: soy la mujer que ya lo recibe. Soy la mujer que ya lo recibe. Soy la mujer que ya lo recibe."
 [2:21–2:28] REVELACIÓN: "El cheque no trae el dinero. Te cambia a ti, y tú traes el dinero."
-[2:28–2:33] COMENTA ✂️: "Si quieres que te guíe, comenta ADN y te mando el link."
-[2:33–2:40] CTA: "En ADN Millonario trabajamos los programas de dinero que heredaste para activar tu frecuencia de abundancia."</t>
+[2:28–2:33] CIERRE: "Guárdalo y sígueme: mañana te enseño a bajarle la velocidad a tu mente."</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1334,17 +1333,17 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>ADN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>ADN Millonario · $750</t>
+          <t>— sin venta (semana foco: Querida Ansiedad)</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>Jim Carrey se escribió un cheque de 10 millones antes de tener éxito 🧾 Te cuento las 3 partes que casi nadie hace. Comenta ADN y te mando el link 👇
+          <t>Jim Carrey se escribió un cheque de 10 millones antes de tener éxito 🧾 Te cuento las 3 partes que casi nadie hace. Guárdalo y sígueme 👇
 #mabradiante #dinero #abundancia #hackeatumente #mty</t>
         </is>
       </c>
@@ -1705,7 +1704,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -1748,8 +1747,7 @@
 [1:02–1:22] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: qué hacías tú en las noches cuando tu mente no te dejaba dormir]"
 [1:22–2:06] HACKEO (hazlo conmigo) ✂️: "Hoy, antes de dormir: 10 minutos escribiendo sin parar lo que sientes, no lo que tienes que hacer. No corrijas nada. Cuando termines, cierra la libreta y di: lo solté en el papel, ya no lo cargo en el cuerpo. Repite conmigo: lo solté en el papel, ya no lo cargo en el cuerpo. Lo solté en el papel, ya no lo cargo en el cuerpo."
 [2:06–2:13] REVELACIÓN: "Lo que no se expresa se queda dando vueltas. Lo que escribes deja de cargarte."
-[2:13–2:19] COMENTA ✂️: "Si tu mente no te deja dormir, comenta DORMIR y te mando el link."
-[2:19–2:27] CTA: "En Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad a tu mente."</t>
+[2:13–2:19] CIERRE · VENTA: "Si tu mente no te deja dormir, en Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad. El link está en mi perfil."</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
@@ -1765,17 +1763,17 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>DORMIR</t>
+          <t>— (el link está en mi perfil)</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Querida Ansiedad · $399</t>
+          <t>Querida Ansiedad · $399 (semana foco)</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr">
         <is>
-          <t>15 minutos de escritura que calman tu mente ✍️ Lo estudió la Universidad de Texas. Te digo cómo hacerlo hoy. Comenta DORMIR y te mando el link 👇
+          <t>15 minutos de escritura que calman tu mente ✍️ Lo estudió la Universidad de Texas. Te digo cómo hacerlo hoy. El link está en mi perfil 👆
 #mabradiante #ansiedad #calmamental #hackeatumente #mty</t>
         </is>
       </c>
@@ -2179,8 +2177,7 @@
 [1:05–1:25] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: una vez que te hiciste chiquita frente a alguien y qué habría hecho tu versión fuerte]"
 [1:25–2:03] HACKEO (hazlo conmigo) ✂️: "Ponle nombre a tu versión que ya no ruega. Hoy, antes de responder un mensaje, pregúntate: ¿qué haría ella? Y responde desde ahí. Repite conmigo: yo elijo desde mi valor, no desde mi miedo. Yo elijo desde mi valor, no desde mi miedo. Yo elijo desde mi valor, no desde mi miedo."
 [2:03–2:10] REVELACIÓN: "No necesitas convertirte en otra persona. Necesitas permiso para ser la versión que ya existe en ti."
-[2:10–2:16] COMENTA ✂️: "Si quieres crear la tuya, comenta ALTER EGO y te mando el link."
-[2:16–2:23] CTA: "En Crea y Activa tu Alter Ego te guío paso a paso para instalar esa identidad."</t>
+[2:10–2:16] CIERRE: "Guárdalo y sígueme para más hackeos."</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -2196,17 +2193,17 @@
       </c>
       <c r="M10" s="12" t="inlineStr">
         <is>
-          <t>ALTER EGO</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>Crea y Activa tu Alter Ego · $599</t>
+          <t>— sin venta (semana foco: Querida Ansiedad)</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Beyoncé tenía un alter ego: Sasha Fierce 🔥 ¿Y tú? 3 cosas que haría tu versión fuerte en el amor. Comenta ALTER EGO y te mando el link 👇
+          <t>Beyoncé tenía un alter ego: Sasha Fierce 🔥 ¿Y tú? 3 cosas que haría tu versión fuerte en el amor. Guárdalo y sígueme 👇
 #mabradiante #relaciones #amorpropio #dependenciaemocional #mty</t>
         </is>
       </c>
@@ -2610,8 +2607,7 @@
 [1:03–1:23] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: un momento difícil que hoy entiendes que te llevó a donde estás]"
 [1:23–1:59] HACKEO (hazlo conmigo) ✂️: "Dibuja una línea en una hoja. Pon 5 momentos clave de tu vida, buenos y difíciles. Únelos. Y pregúntate: ¿hacia dónde apuntan? Repite conmigo: nada de lo que viví fue en vano. Nada de lo que viví fue en vano. Nada de lo que viví fue en vano."
 [1:59–2:04] REVELACIÓN: "Tu vida no está desordenada. Todavía no has visto el dibujo completo."
-[2:04–2:10] COMENTA ✂️: "Si quieres un mapa para tu despertar, comenta DESPIERTA y te mando el link."
-[2:10–2:17] CTA: "En DESPIERTA te acompaño en los primeros pasos de tu despertar con un mapa claro."</t>
+[2:04–2:10] CIERRE: "Guárdalo y sígueme para más hackeos de consciencia."</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
@@ -2627,17 +2623,17 @@
       </c>
       <c r="M13" s="15" t="inlineStr">
         <is>
-          <t>DESPIERTA</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" s="15" t="inlineStr">
         <is>
-          <t>DESPIERTA · $499</t>
+          <t>— sin venta (semana foco: Querida Ansiedad)</t>
         </is>
       </c>
       <c r="O13" s="15" t="inlineStr">
         <is>
-          <t>Lo que Steve Jobs dijo sobre unir los puntos 🔗 y por qué hoy no le encuentras sentido a tu vida. Comenta DESPIERTA y te mando el link 👇
+          <t>Lo que Steve Jobs dijo sobre unir los puntos 🔗 y por qué hoy no le encuentras sentido a tu vida. Guárdalo y sígueme 👇
 #mabradiante #despertardeconciencia #espiritualidad #salirdelamatrix #mty</t>
         </is>
       </c>
@@ -2998,7 +2994,7 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -3041,8 +3037,7 @@
 [0:59–1:19] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: tu momento de agotamiento y qué te hizo parar]"
 [1:19–1:51] HACKEO (hazlo conmigo) ✂️: "Elige hoy una sola cosa que vas a dejar de hacer esta semana. Solo una. Escríbela y avísale a alguien. Repite conmigo: dejar de hacer también es avanzar. Dejar de hacer también es avanzar. Dejar de hacer también es avanzar."
 [1:51–1:54] REVELACIÓN: "No necesitas más energía. Necesitas dejar de fugarla."
-[1:54–2:00] COMENTA ✂️: "Si quieres salir de la alerta, comenta APAGAR y te mando el link."
-[2:00–2:07] CTA: "En Apaga el Modo Supervivencia te doy el protocolo para salir de la alerta paso a paso."</t>
+[1:54–2:00] CIERRE · VENTA: "Si tu cuerpo está en alerta y tu mente no se apaga ni cuando duermes, en Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad. El link está en mi perfil."</t>
         </is>
       </c>
       <c r="K16" s="18" t="inlineStr">
@@ -3058,17 +3053,17 @@
       </c>
       <c r="M16" s="18" t="inlineStr">
         <is>
-          <t>APAGAR</t>
+          <t>— (el link está en mi perfil)</t>
         </is>
       </c>
       <c r="N16" s="18" t="inlineStr">
         <is>
-          <t>Apaga el Modo Supervivencia · $750</t>
+          <t>Querida Ansiedad · $399 (semana foco)</t>
         </is>
       </c>
       <c r="O16" s="18" t="inlineStr">
         <is>
-          <t>La OMS ya le puso nombre a tu agotamiento 🔋 Estas son las 3 señales. Comenta APAGAR y te mando el link 👇
+          <t>La OMS ya le puso nombre a tu agotamiento 🔋 Estas son las 3 señales. El link está en mi perfil 👆
 #mabradiante #energia #modosupervivencia #ritual #mty</t>
         </is>
       </c>
@@ -3472,8 +3467,7 @@
 [1:00–1:20] TU HISTORIA: "[TU HISTORIA REAL, 15–20 s: qué significaba fallar en tu casa cuando eras niña]"
 [1:20–1:53] HACKEO (hazlo conmigo) ✂️: "Hoy responde tú la pregunta: ¿en qué fallé esta semana y qué aprendí? Escríbelo sin juzgarte. Repite conmigo: fallar es la prueba de que lo intenté. Fallar es la prueba de que lo intenté. Fallar es la prueba de que lo intenté."
 [1:53–2:00] REVELACIÓN: "La creencia más peligrosa es la que no sabes que tienes. Y casi siempre es sobre fallar."
-[2:00–2:07] COMENTA ✂️: "Si quieres hackear tus creencias de raíz, comenta NIVEL 1 y te mando el link."
-[2:07–2:14] CTA: "En el Nivel 1 de Las Fórmulas Cuánticas hackeamos las creencias que no sabes que tienes."</t>
+[2:00–2:07] CIERRE: "Guárdalo y sígueme: mañana cerramos la semana juntas."</t>
         </is>
       </c>
       <c r="K19" s="21" t="inlineStr">
@@ -3489,17 +3483,17 @@
       </c>
       <c r="M19" s="21" t="inlineStr">
         <is>
-          <t>NIVEL 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N19" s="21" t="inlineStr">
         <is>
-          <t>Nivel 1 DESPERTAR · $2,000</t>
+          <t>— sin venta (semana foco: Querida Ansiedad)</t>
         </is>
       </c>
       <c r="O19" s="21" t="inlineStr">
         <is>
-          <t>La pregunta que el papá de Sara Blakely le hacía cada semana 💡 y las 3 creencias que te frenan. Comenta NIVEL 1 y te mando el link 👇
+          <t>La pregunta que el papá de Sara Blakely le hacía cada semana 💡 y las 3 creencias que te frenan. Guárdalo y sígueme 👇
 #mabradiante #metas #leydeatraccion #decreto #mty</t>
         </is>
       </c>
@@ -4295,12 +4289,12 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Si quieres que te guíe, comenta ADN y te mando el link.</t>
+          <t>Guárdalo y sígueme: mañana te enseño a bajarle la velocidad a tu mente.</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>En ADN Millonario trabajamos los programas de dinero que heredaste para activar tu frecuencia de abundancia.</t>
+          <t>— sin venta</t>
         </is>
       </c>
     </row>
@@ -4490,12 +4484,12 @@
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>Si tu mente no te deja dormir, comenta DORMIR y te mando el link.</t>
+          <t>Si tu mente no te deja dormir, en Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad. El link está en mi perfil.</t>
         </is>
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>En Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad a tu mente.</t>
+          <t>(venta incluida en el cierre)</t>
         </is>
       </c>
     </row>
@@ -4685,12 +4679,12 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>Si quieres crear la tuya, comenta ALTER EGO y te mando el link.</t>
+          <t>Guárdalo y sígueme para más hackeos.</t>
         </is>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>En Crea y Activa tu Alter Ego te guío paso a paso para instalar esa identidad.</t>
+          <t>— sin venta</t>
         </is>
       </c>
     </row>
@@ -4880,12 +4874,12 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>Si quieres un mapa para tu despertar, comenta DESPIERTA y te mando el link.</t>
+          <t>Guárdalo y sígueme para más hackeos de consciencia.</t>
         </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
-          <t>En DESPIERTA te acompaño en los primeros pasos de tu despertar con un mapa claro.</t>
+          <t>— sin venta</t>
         </is>
       </c>
     </row>
@@ -5075,12 +5069,12 @@
       </c>
       <c r="K16" s="18" t="inlineStr">
         <is>
-          <t>Si quieres salir de la alerta, comenta APAGAR y te mando el link.</t>
+          <t>Si tu cuerpo está en alerta y tu mente no se apaga ni cuando duermes, en Querida Ansiedad te doy la auditoría mental y los audios para bajarle la velocidad. El link está en mi perfil.</t>
         </is>
       </c>
       <c r="L16" s="18" t="inlineStr">
         <is>
-          <t>En Apaga el Modo Supervivencia te doy el protocolo para salir de la alerta paso a paso.</t>
+          <t>(venta incluida en el cierre)</t>
         </is>
       </c>
     </row>
@@ -5270,12 +5264,12 @@
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
-          <t>Si quieres hackear tus creencias de raíz, comenta NIVEL 1 y te mando el link.</t>
+          <t>Guárdalo y sígueme: mañana cerramos la semana juntas.</t>
         </is>
       </c>
       <c r="L19" s="21" t="inlineStr">
         <is>
-          <t>En el Nivel 1 de Las Fórmulas Cuánticas hackeamos las creencias que no sabes que tienes.</t>
+          <t>— sin venta</t>
         </is>
       </c>
     </row>
@@ -5578,7 +5572,7 @@
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Publicar a su hora y responder los comentarios con la palabra clave (con el link si es pieza de venta).</t>
+          <t>Publicar a su hora (las 2 piezas de venta, martes y viernes, a las 19:30) y responder comentarios. Esta semana solo se vende Querida Ansiedad: el link está en tu perfil (Linktree, primer botón).</t>
         </is>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -13708,8 +13702,8 @@
   <mergeCells count="18">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A23:F23"/>

</xml_diff>